<commit_message>
Implementar 8 graficas + normalizar tamaño AB#58
</commit_message>
<xml_diff>
--- a/docs/Horas proyecto estadistica.xlsx
+++ b/docs/Horas proyecto estadistica.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Trabajo_final\AppClientesEstadistica\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0751B9E8-D6F6-4AE6-9881-43DEEDFE7B29}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD816F67-EB90-4F0F-BED5-EC26B077A074}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="12315" windowHeight="7980" xr2:uid="{75DE17B3-81B2-44DB-AF0F-61090BDD4A63}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="41">
   <si>
     <t>Roberto</t>
   </si>
@@ -266,16 +266,45 @@
   </si>
   <si>
     <t xml:space="preserve">
-- Tener todo hosteado
-- Tener una versión entregable
-- Tener BBDD definitiva
-- Definir conexiones con resto equipo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
 Roberto =&gt; Login back y front
 Irantzu + Carlos + Roberto =&gt; Menu + Funcionalidades + Datos
 Sergio =&gt; Registro + DevOps</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Tener todo hosteado</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFFFF00"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+- Tener una versión entregable
+- Tener BBDD definitiva
+- Definir conexiones con resto equipo
+Sergio =&gt; Apartado display graficas estadistica</t>
+    </r>
+  </si>
+  <si>
+    <t>- Implementar 8 graficas máx
+- Normalizar tamaño graficas</t>
   </si>
 </sst>
 </file>
@@ -692,7 +721,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -766,6 +795,30 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1218,7 +1271,7 @@
     <col min="14" max="14" width="3.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="20" t="s">
         <v>14</v>
       </c>
@@ -1228,8 +1281,8 @@
       <c r="F1" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="21"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="27"/>
       <c r="I1" s="20" t="s">
         <v>16</v>
       </c>
@@ -1241,14 +1294,14 @@
       <c r="M1" s="21"/>
       <c r="N1" s="22"/>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="23"/>
       <c r="C2" s="24"/>
       <c r="D2" s="24"/>
       <c r="E2" s="25"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="25"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="30"/>
       <c r="I2" s="23"/>
       <c r="J2" s="24"/>
       <c r="K2" s="25"/>
@@ -1256,14 +1309,14 @@
       <c r="M2" s="24"/>
       <c r="N2" s="25"/>
     </row>
-    <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="23"/>
       <c r="C3" s="24"/>
       <c r="D3" s="24"/>
       <c r="E3" s="25"/>
-      <c r="F3" s="23"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="25"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="33"/>
       <c r="I3" s="23"/>
       <c r="J3" s="24"/>
       <c r="K3" s="25"/>
@@ -1327,7 +1380,9 @@
       <c r="F5" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="10"/>
+      <c r="G5" s="16" t="s">
+        <v>40</v>
+      </c>
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
@@ -1409,238 +1464,238 @@
       <c r="N8" s="14"/>
     </row>
     <row r="9" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="26" t="s">
+      <c r="C9" s="43"/>
+      <c r="D9" s="43"/>
+      <c r="E9" s="44"/>
+      <c r="F9" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="26" t="s">
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="J9" s="27"/>
-      <c r="K9" s="27"/>
-      <c r="L9" s="26" t="s">
+      <c r="J9" s="35"/>
+      <c r="K9" s="35"/>
+      <c r="L9" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="M9" s="27"/>
-      <c r="N9" s="27"/>
+      <c r="M9" s="35"/>
+      <c r="N9" s="35"/>
     </row>
     <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="45" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="46"/>
+      <c r="D10" s="46"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="46" t="s">
-        <v>38</v>
-      </c>
-      <c r="G10" s="38"/>
-      <c r="H10" s="38"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="29"/>
-      <c r="K10" s="29"/>
-      <c r="L10" s="28"/>
-      <c r="M10" s="29"/>
-      <c r="N10" s="29"/>
+      <c r="G10" s="46"/>
+      <c r="H10" s="46"/>
+      <c r="I10" s="36"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="37"/>
+      <c r="L10" s="36"/>
+      <c r="M10" s="37"/>
+      <c r="N10" s="37"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="40"/>
-      <c r="C11" s="41"/>
-      <c r="D11" s="41"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="40"/>
-      <c r="G11" s="41"/>
-      <c r="H11" s="41"/>
-      <c r="I11" s="30"/>
-      <c r="J11" s="31"/>
-      <c r="K11" s="31"/>
-      <c r="L11" s="30"/>
-      <c r="M11" s="31"/>
-      <c r="N11" s="31"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="49"/>
+      <c r="D11" s="49"/>
+      <c r="E11" s="50"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="49"/>
+      <c r="H11" s="49"/>
+      <c r="I11" s="38"/>
+      <c r="J11" s="39"/>
+      <c r="K11" s="39"/>
+      <c r="L11" s="38"/>
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="40"/>
-      <c r="C12" s="41"/>
-      <c r="D12" s="41"/>
-      <c r="E12" s="42"/>
-      <c r="F12" s="40"/>
-      <c r="G12" s="41"/>
-      <c r="H12" s="41"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="31"/>
-      <c r="K12" s="31"/>
-      <c r="L12" s="30"/>
-      <c r="M12" s="31"/>
-      <c r="N12" s="31"/>
+      <c r="B12" s="48"/>
+      <c r="C12" s="49"/>
+      <c r="D12" s="49"/>
+      <c r="E12" s="50"/>
+      <c r="F12" s="48"/>
+      <c r="G12" s="49"/>
+      <c r="H12" s="49"/>
+      <c r="I12" s="38"/>
+      <c r="J12" s="39"/>
+      <c r="K12" s="39"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="39"/>
+      <c r="N12" s="39"/>
     </row>
     <row r="13" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="40"/>
-      <c r="C13" s="41"/>
-      <c r="D13" s="41"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="40"/>
-      <c r="G13" s="41"/>
-      <c r="H13" s="41"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="31"/>
-      <c r="L13" s="30"/>
-      <c r="M13" s="31"/>
-      <c r="N13" s="31"/>
+      <c r="B13" s="48"/>
+      <c r="C13" s="49"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="48"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="49"/>
+      <c r="I13" s="38"/>
+      <c r="J13" s="39"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="38"/>
+      <c r="M13" s="39"/>
+      <c r="N13" s="39"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="40"/>
-      <c r="C14" s="41"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="42"/>
-      <c r="F14" s="40"/>
-      <c r="G14" s="41"/>
-      <c r="H14" s="41"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="31"/>
-      <c r="K14" s="31"/>
-      <c r="L14" s="30"/>
-      <c r="M14" s="31"/>
-      <c r="N14" s="31"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="49"/>
+      <c r="D14" s="49"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="49"/>
+      <c r="I14" s="38"/>
+      <c r="J14" s="39"/>
+      <c r="K14" s="39"/>
+      <c r="L14" s="38"/>
+      <c r="M14" s="39"/>
+      <c r="N14" s="39"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="40"/>
-      <c r="C15" s="41"/>
-      <c r="D15" s="41"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="41"/>
-      <c r="H15" s="41"/>
-      <c r="I15" s="30"/>
-      <c r="J15" s="31"/>
-      <c r="K15" s="31"/>
-      <c r="L15" s="30"/>
-      <c r="M15" s="31"/>
-      <c r="N15" s="31"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="49"/>
+      <c r="D15" s="49"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="49"/>
+      <c r="I15" s="38"/>
+      <c r="J15" s="39"/>
+      <c r="K15" s="39"/>
+      <c r="L15" s="38"/>
+      <c r="M15" s="39"/>
+      <c r="N15" s="39"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="40"/>
-      <c r="C16" s="41"/>
-      <c r="D16" s="41"/>
-      <c r="E16" s="42"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="41"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="31"/>
-      <c r="K16" s="31"/>
-      <c r="L16" s="30"/>
-      <c r="M16" s="31"/>
-      <c r="N16" s="31"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="49"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="49"/>
+      <c r="I16" s="38"/>
+      <c r="J16" s="39"/>
+      <c r="K16" s="39"/>
+      <c r="L16" s="38"/>
+      <c r="M16" s="39"/>
+      <c r="N16" s="39"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B17" s="40"/>
-      <c r="C17" s="41"/>
-      <c r="D17" s="41"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="41"/>
-      <c r="H17" s="41"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="31"/>
-      <c r="L17" s="30"/>
-      <c r="M17" s="31"/>
-      <c r="N17" s="31"/>
+      <c r="B17" s="48"/>
+      <c r="C17" s="49"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="49"/>
+      <c r="H17" s="49"/>
+      <c r="I17" s="38"/>
+      <c r="J17" s="39"/>
+      <c r="K17" s="39"/>
+      <c r="L17" s="38"/>
+      <c r="M17" s="39"/>
+      <c r="N17" s="39"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B18" s="40"/>
-      <c r="C18" s="41"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="42"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="41"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
-      <c r="L18" s="30"/>
-      <c r="M18" s="31"/>
-      <c r="N18" s="31"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="49"/>
+      <c r="I18" s="38"/>
+      <c r="J18" s="39"/>
+      <c r="K18" s="39"/>
+      <c r="L18" s="38"/>
+      <c r="M18" s="39"/>
+      <c r="N18" s="39"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B19" s="40"/>
-      <c r="C19" s="41"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="41"/>
-      <c r="H19" s="41"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="31"/>
-      <c r="L19" s="30"/>
-      <c r="M19" s="31"/>
-      <c r="N19" s="31"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="49"/>
+      <c r="D19" s="49"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="49"/>
+      <c r="H19" s="49"/>
+      <c r="I19" s="38"/>
+      <c r="J19" s="39"/>
+      <c r="K19" s="39"/>
+      <c r="L19" s="38"/>
+      <c r="M19" s="39"/>
+      <c r="N19" s="39"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B20" s="40"/>
-      <c r="C20" s="41"/>
-      <c r="D20" s="41"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="40"/>
-      <c r="G20" s="41"/>
-      <c r="H20" s="41"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="30"/>
-      <c r="M20" s="31"/>
-      <c r="N20" s="31"/>
+      <c r="B20" s="48"/>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="49"/>
+      <c r="H20" s="49"/>
+      <c r="I20" s="38"/>
+      <c r="J20" s="39"/>
+      <c r="K20" s="39"/>
+      <c r="L20" s="38"/>
+      <c r="M20" s="39"/>
+      <c r="N20" s="39"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B21" s="40"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="41"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="41"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="31"/>
-      <c r="K21" s="31"/>
-      <c r="L21" s="30"/>
-      <c r="M21" s="31"/>
-      <c r="N21" s="31"/>
+      <c r="B21" s="48"/>
+      <c r="C21" s="49"/>
+      <c r="D21" s="49"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="48"/>
+      <c r="G21" s="49"/>
+      <c r="H21" s="49"/>
+      <c r="I21" s="38"/>
+      <c r="J21" s="39"/>
+      <c r="K21" s="39"/>
+      <c r="L21" s="38"/>
+      <c r="M21" s="39"/>
+      <c r="N21" s="39"/>
     </row>
     <row r="22" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="43"/>
-      <c r="C22" s="44"/>
-      <c r="D22" s="44"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="44"/>
-      <c r="H22" s="44"/>
-      <c r="I22" s="32"/>
-      <c r="J22" s="33"/>
-      <c r="K22" s="33"/>
-      <c r="L22" s="32"/>
-      <c r="M22" s="33"/>
-      <c r="N22" s="33"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="52"/>
+      <c r="E22" s="53"/>
+      <c r="F22" s="51"/>
+      <c r="G22" s="52"/>
+      <c r="H22" s="52"/>
+      <c r="I22" s="40"/>
+      <c r="J22" s="41"/>
+      <c r="K22" s="41"/>
+      <c r="L22" s="40"/>
+      <c r="M22" s="41"/>
+      <c r="N22" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>